<commit_message>
Table Formatted and Monthly Target or Goal is Calculated
</commit_message>
<xml_diff>
--- a/Day 6/Monthly_Students_Course_Fee.xlsx
+++ b/Day 6/Monthly_Students_Course_Fee.xlsx
@@ -1,40 +1,140 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F483BC3-5D4B-4084-A0AA-CCA16D437030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Courses Fee</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>Monthly Sale</t>
+  </si>
+  <si>
+    <t>Total Sales From Jan to June</t>
+  </si>
+  <si>
+    <t>Yearly Target</t>
+  </si>
+  <si>
+    <t>Remaining Target</t>
+  </si>
+  <si>
+    <t>Remaining Months</t>
+  </si>
+  <si>
+    <t>Monthly Target</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,85 +146,36 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="3">
+    <cellStyle name="Accent3" xfId="2" builtinId="37"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,110 +463,156 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="1"/>
+    <col min="2" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.77734375" customWidth="1"/>
+    <col min="8" max="8" width="20.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Students</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Courses Fee</t>
-        </is>
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="4">
+        <v>3000000</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2">
         <v>40</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2">
         <v>5000</v>
       </c>
+      <c r="D2" s="2">
+        <f>B2*C2</f>
+        <v>200000</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="4">
+        <f>SUM(D2:D7)</f>
+        <v>1575000</v>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>February</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2">
         <v>45</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2">
         <v>5000</v>
       </c>
+      <c r="D3" s="2">
+        <f t="shared" ref="D3:D13" si="0">B3*C3</f>
+        <v>225000</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="5">
+        <f>H1-H2</f>
+        <v>1425000</v>
+      </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2">
         <v>50</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2">
         <v>5000</v>
       </c>
+      <c r="D4" s="2">
+        <f t="shared" si="0"/>
+        <v>250000</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="5">
+        <v>6</v>
+      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>April</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2">
         <v>55</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2">
         <v>5000</v>
       </c>
+      <c r="D5" s="2">
+        <f t="shared" si="0"/>
+        <v>275000</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="5">
+        <f>H3/H4</f>
+        <v>237500</v>
+      </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2">
         <v>60</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2">
         <v>5000</v>
       </c>
+      <c r="D6" s="2">
+        <f t="shared" si="0"/>
+        <v>300000</v>
+      </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>June</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2">
         <v>65</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2">
         <v>5000</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" si="0"/>
+        <v>325000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
What if Goal Seek Analycis is done for the month of August
</commit_message>
<xml_diff>
--- a/Day 6/Monthly_Students_Course_Fee.xlsx
+++ b/Day 6/Monthly_Students_Course_Fee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F483BC3-5D4B-4084-A0AA-CCA16D437030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B47CC9A-37C6-4D2C-BA77-7B5F64907EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Month</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Monthly Sale</t>
   </si>
   <si>
-    <t>Total Sales From Jan to June</t>
-  </si>
-  <si>
     <t>Yearly Target</t>
   </si>
   <si>
@@ -77,6 +74,27 @@
   </si>
   <si>
     <t>Monthly Target</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>December</t>
+  </si>
+  <si>
+    <t>Total Sales From Jan to July</t>
   </si>
 </sst>
 </file>
@@ -87,7 +105,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +137,12 @@
     <font>
       <sz val="16"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -464,12 +488,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
     <col min="6" max="6" width="34.77734375" customWidth="1"/>
     <col min="8" max="8" width="20.21875" customWidth="1"/>
   </cols>
@@ -488,7 +513,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" s="4">
         <v>3000000</v>
@@ -509,11 +534,11 @@
         <v>200000</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H2" s="4">
-        <f>SUM(D2:D7)</f>
-        <v>1575000</v>
+        <f>SUM(D2:D8)</f>
+        <v>1775000</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
@@ -531,11 +556,11 @@
         <v>225000</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H3" s="5">
         <f>H1-H2</f>
-        <v>1425000</v>
+        <v>1225000</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.4">
@@ -553,10 +578,10 @@
         <v>250000</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.4">
@@ -574,11 +599,11 @@
         <v>275000</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="5">
         <f>H3/H4</f>
-        <v>237500</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.3">
@@ -611,7 +636,90 @@
         <v>325000</v>
       </c>
     </row>
+    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" si="0"/>
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="2">
+        <v>49</v>
+      </c>
+      <c r="C9" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" si="0"/>
+        <v>245000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2">
+        <v>5000</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>